<commit_message>
feat(db,models,api): defer series.is_default (ADR 0027)
Remove the series.is_default column. It was an unenforced (no partial-unique),
advisory boolean, absent from the admin surface, that disambiguated nothing while
every (concept, geography) slice carried a single series. Defer the
default-reading marker until a real multi-series slice needs it (cheap to re-add;
consistent with ADR 0025's loose-first stance). Reverses the ADR 0025 §1 decision
to materialize indicator_variants.is_default on series.

- migration 0021 drops the column (downgrade re-adds it at its 0019 shape)
- drop it from the Series model, SeriesBase/SeriesUpdate schemas, the bootstrap
  RawSeriesSpec + payload, and the list_series `is_default` query filter
- db_er.txt (canonical) and CONTEXT.md mark the default reading as deferred
- tests: series has no is_default at head; drop the default-filter API case and
  the bootstrap one-default-per-slice test

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/schema/category_taxonomy.xlsx
+++ b/docs/schema/category_taxonomy.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Taxonomy (L1-L2-L3)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seed rows (flat)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review findings" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open questions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Taxonomy (L1-L2-L3)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Seed rows (flat)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Review findings" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Open questions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Taxonomy (L1-L2-L3)'!$A$1:$F$1</definedName>

</xml_diff>